<commit_message>
PMO: AI pre-fill Facebook Groups (5) + KOL creators (7) with notes, business confirms/adds/removes
</commit_message>
<xml_diff>
--- a/PMO/02_阶段二_数据采集落地/业务协作_待业务填写事项.xlsx
+++ b/PMO/02_阶段二_数据采集落地/业务协作_待业务填写事项.xlsx
@@ -440,11 +440,11 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,74 +460,154 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>是否公开</t>
+          <t>主题/垂类</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>主题/垂类</t>
+          <t>AI备注</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>业务确认</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exclusively Pumping Mamas - Education &amp; Support Group</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/1574856819503023/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>排奶/泵奶支持</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>教育+支持型，活跃度高，S1 用户讨论核心群</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Exclusive Pumping: Breastfeeding Without Nursing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/groups/EP.BWN/</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>排奶/泵奶支持</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>经典排奶大群，跨地区</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Wearable Pump Paperweight Prevention</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>URL 待社媒团队补充</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>可穿戴泵 troubleshooting</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IBCLC Jessica Anderson 运营，可穿戴泵专业讨论</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Breastfeeding Support Group for Black Moms</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>URL 待社媒团队补充</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>母乳支持</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>约 9.1 万成员大群</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pumping Mamas: breastfeeding support for working moms</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>URL 待社媒团队补充</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>职场泵奶</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>职场妈妈泵奶场景，与 Momcozy 目标人群重合</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
@@ -541,14 +621,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,70 +649,196 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>是否已合作</t>
+          <t>AI备注</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>业务确认</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Allison Tolman / New Little Life</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>泵奶器测评 IBCLC</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>头部泵奶器专家，万粉级，可做专家背书/Pitch</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr"/>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Jessica Anderson / Genuine Lactation</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Instagram+FB</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>可穿戴泵 IBCLC</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>可穿戴泵专业测评，运营 Wearable Pump Paperweight 群</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Katie Clark / The Breastfeeding Mama</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>YouTube</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>泵奶器 IBCLC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>IBCLC 推荐类内容，6.7K+ 播放</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr"/>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Carisa Myers / The Milk Effect</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>泵奶器 RN IBCLC</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>测评 30+ 泵，100 分评分体系，无赞助</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Allison Banfield / Pumping Milk</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>YouTube+Blog</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Momcozy 测评</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Momcozy 全系列测评（M5/M6/M9/V1 Pro），可合作</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tamari Jacob / @onewiththepump</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Instagram/Threads</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>排奶/泵奶</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>16.9K 粉丝，排奶教育</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>maxinesanz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>泵奶器测评</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>新手妈妈泵奶测评，#momcozy #spectra</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>